<commit_message>
data(snapshots): weekly scores 2026-10-31
</commit_message>
<xml_diff>
--- a/snapshots/scores_2026.xlsx
+++ b/snapshots/scores_2026.xlsx
@@ -10,7 +10,7 @@
     <sheet name="2026" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026'!$A$1:$Y$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026'!$A$1:$Y$51</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y26"/>
+  <dimension ref="A1:Y51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2905,8 +2905,2321 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" s="2" t="n">
+        <v>46325</v>
+      </c>
+      <c r="F27" t="n">
+        <v>344.63</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="H27" t="n">
+        <v>755.72</v>
+      </c>
+      <c r="I27" t="n">
+        <v>46.5</v>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L27" t="n">
+        <v>35.6</v>
+      </c>
+      <c r="M27" t="n">
+        <v>57.5</v>
+      </c>
+      <c r="N27" t="n">
+        <v>344.63</v>
+      </c>
+      <c r="O27" t="n">
+        <v>1.069</v>
+      </c>
+      <c r="P27" t="n">
+        <v>39.52179</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>36.068707</v>
+      </c>
+      <c r="R27" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="S27" t="n">
+        <v>0.003134</v>
+      </c>
+      <c r="T27" t="n">
+        <v>0.287</v>
+      </c>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="V27" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="W27" t="n">
+        <v>0.0498</v>
+      </c>
+      <c r="X27" t="inlineStr">
+        <is>
+          <t>fred</t>
+        </is>
+      </c>
+      <c r="Y27" t="inlineStr">
+        <is>
+          <t>e95d114</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" s="2" t="n">
+        <v>46325</v>
+      </c>
+      <c r="F28" t="n">
+        <v>521.91</v>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="H28" t="n">
+        <v>755.72</v>
+      </c>
+      <c r="I28" t="n">
+        <v>47.4</v>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L28" t="n">
+        <v>35.8</v>
+      </c>
+      <c r="M28" t="n">
+        <v>59</v>
+      </c>
+      <c r="N28" t="n">
+        <v>521.91</v>
+      </c>
+      <c r="O28" t="n">
+        <v>1.099</v>
+      </c>
+      <c r="P28" t="n">
+        <v>27.239561</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>21.618698</v>
+      </c>
+      <c r="R28" t="n">
+        <v>3.92</v>
+      </c>
+      <c r="S28" t="n">
+        <v>0.007511</v>
+      </c>
+      <c r="T28" t="n">
+        <v>0.323</v>
+      </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="V28" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="W28" t="n">
+        <v>0.0498</v>
+      </c>
+      <c r="X28" t="inlineStr">
+        <is>
+          <t>fred</t>
+        </is>
+      </c>
+      <c r="Y28" t="inlineStr">
+        <is>
+          <t>e95d114</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" s="2" t="n">
+        <v>46325</v>
+      </c>
+      <c r="F29" t="n">
+        <v>279.84</v>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="H29" t="n">
+        <v>755.72</v>
+      </c>
+      <c r="I29" t="n">
+        <v>37.4</v>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L29" t="n">
+        <v>33.8</v>
+      </c>
+      <c r="M29" t="n">
+        <v>41</v>
+      </c>
+      <c r="N29" t="n">
+        <v>279.84</v>
+      </c>
+      <c r="O29" t="n">
+        <v>1.211</v>
+      </c>
+      <c r="P29" t="n">
+        <v>14.613055</v>
+      </c>
+      <c r="Q29" t="n">
+        <v>18.485123</v>
+      </c>
+      <c r="R29" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="S29" t="n">
+        <v>0.003145</v>
+      </c>
+      <c r="T29" t="n">
+        <v>-0.253</v>
+      </c>
+      <c r="U29" t="inlineStr">
+        <is>
+          <t>Communication Services</t>
+        </is>
+      </c>
+      <c r="V29" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="W29" t="n">
+        <v>0.0498</v>
+      </c>
+      <c r="X29" t="inlineStr">
+        <is>
+          <t>fred</t>
+        </is>
+      </c>
+      <c r="Y29" t="inlineStr">
+        <is>
+          <t>e95d114</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" s="2" t="n">
+        <v>46325</v>
+      </c>
+      <c r="F30" t="n">
+        <v>240.35</v>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="H30" t="n">
+        <v>755.72</v>
+      </c>
+      <c r="I30" t="n">
+        <v>48</v>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="L30" t="n">
+        <v>59.6</v>
+      </c>
+      <c r="M30" t="n">
+        <v>36.5</v>
+      </c>
+      <c r="N30" t="n">
+        <v>240.35</v>
+      </c>
+      <c r="O30" t="inlineStr"/>
+      <c r="P30" t="n">
+        <v>19.430073</v>
+      </c>
+      <c r="Q30" t="n">
+        <v>22.804256</v>
+      </c>
+      <c r="R30" t="inlineStr"/>
+      <c r="S30" t="n">
+        <v>0</v>
+      </c>
+      <c r="T30" t="n">
+        <v>-0.031</v>
+      </c>
+      <c r="U30" t="inlineStr">
+        <is>
+          <t>Consumer Cyclical</t>
+        </is>
+      </c>
+      <c r="V30" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="W30" t="n">
+        <v>0.0498</v>
+      </c>
+      <c r="X30" t="inlineStr">
+        <is>
+          <t>fred</t>
+        </is>
+      </c>
+      <c r="Y30" t="inlineStr">
+        <is>
+          <t>e95d114</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" s="2" t="n">
+        <v>46325</v>
+      </c>
+      <c r="F31" t="n">
+        <v>204.64</v>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="H31" t="n">
+        <v>755.72</v>
+      </c>
+      <c r="I31" t="n">
+        <v>33.8</v>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L31" t="n">
+        <v>16</v>
+      </c>
+      <c r="M31" t="n">
+        <v>51.5</v>
+      </c>
+      <c r="N31" t="n">
+        <v>204.64</v>
+      </c>
+      <c r="O31" t="n">
+        <v>2.216</v>
+      </c>
+      <c r="P31" t="n">
+        <v>25.87105</v>
+      </c>
+      <c r="Q31" t="n">
+        <v>12.858633</v>
+      </c>
+      <c r="R31" t="n">
+        <v>1</v>
+      </c>
+      <c r="S31" t="n">
+        <v>0.004887</v>
+      </c>
+      <c r="T31" t="n">
+        <v>1.278</v>
+      </c>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="V31" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="W31" t="n">
+        <v>0.0498</v>
+      </c>
+      <c r="X31" t="inlineStr">
+        <is>
+          <t>fred</t>
+        </is>
+      </c>
+      <c r="Y31" t="inlineStr">
+        <is>
+          <t>e95d114</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" s="2" t="n">
+        <v>46325</v>
+      </c>
+      <c r="F32" t="n">
+        <v>614.99</v>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="H32" t="n">
+        <v>755.72</v>
+      </c>
+      <c r="I32" t="n">
+        <v>34</v>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L32" t="n">
+        <v>33.1</v>
+      </c>
+      <c r="M32" t="n">
+        <v>35</v>
+      </c>
+      <c r="N32" t="n">
+        <v>614.99</v>
+      </c>
+      <c r="O32" t="n">
+        <v>1.185</v>
+      </c>
+      <c r="P32" t="n">
+        <v>20.982258</v>
+      </c>
+      <c r="Q32" t="n">
+        <v>17.2809</v>
+      </c>
+      <c r="R32" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="S32" t="n">
+        <v>0.003415</v>
+      </c>
+      <c r="T32" t="n">
+        <v>2.648</v>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>Communication Services</t>
+        </is>
+      </c>
+      <c r="V32" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="W32" t="n">
+        <v>0.0498</v>
+      </c>
+      <c r="X32" t="inlineStr">
+        <is>
+          <t>fred</t>
+        </is>
+      </c>
+      <c r="Y32" t="inlineStr">
+        <is>
+          <t>e95d114</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>JPM</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" s="2" t="n">
+        <v>46325</v>
+      </c>
+      <c r="F33" t="n">
+        <v>337.04</v>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="H33" t="n">
+        <v>755.72</v>
+      </c>
+      <c r="I33" t="n">
+        <v>75.5</v>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L33" t="n">
+        <v>90.5</v>
+      </c>
+      <c r="M33" t="n">
+        <v>60.5</v>
+      </c>
+      <c r="N33" t="n">
+        <v>337.04</v>
+      </c>
+      <c r="O33" t="n">
+        <v>1.015</v>
+      </c>
+      <c r="P33" t="n">
+        <v>14.137584</v>
+      </c>
+      <c r="Q33" t="n">
+        <v>13.201082</v>
+      </c>
+      <c r="R33" t="n">
+        <v>6.6</v>
+      </c>
+      <c r="S33" t="n">
+        <v>0.019582</v>
+      </c>
+      <c r="T33" t="n">
+        <v>0.099</v>
+      </c>
+      <c r="U33" t="inlineStr">
+        <is>
+          <t>Financial Services</t>
+        </is>
+      </c>
+      <c r="V33" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="W33" t="n">
+        <v>0.0498</v>
+      </c>
+      <c r="X33" t="inlineStr">
+        <is>
+          <t>fred</t>
+        </is>
+      </c>
+      <c r="Y33" t="inlineStr">
+        <is>
+          <t>e95d114</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" s="2" t="n">
+        <v>46325</v>
+      </c>
+      <c r="F34" t="n">
+        <v>413.59</v>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="H34" t="n">
+        <v>755.72</v>
+      </c>
+      <c r="I34" t="n">
+        <v>62.4</v>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="L34" t="n">
+        <v>62.7</v>
+      </c>
+      <c r="M34" t="n">
+        <v>62</v>
+      </c>
+      <c r="N34" t="n">
+        <v>413.59</v>
+      </c>
+      <c r="O34" t="n">
+        <v>0.771</v>
+      </c>
+      <c r="P34" t="n">
+        <v>33.570618</v>
+      </c>
+      <c r="Q34" t="n">
+        <v>24.140387</v>
+      </c>
+      <c r="R34" t="n">
+        <v>2.68</v>
+      </c>
+      <c r="S34" t="n">
+        <v>0.00648</v>
+      </c>
+      <c r="T34" t="n">
+        <v>0.219</v>
+      </c>
+      <c r="U34" t="inlineStr">
+        <is>
+          <t>Financial Services</t>
+        </is>
+      </c>
+      <c r="V34" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="W34" t="n">
+        <v>0.0498</v>
+      </c>
+      <c r="X34" t="inlineStr">
+        <is>
+          <t>fred</t>
+        </is>
+      </c>
+      <c r="Y34" t="inlineStr">
+        <is>
+          <t>e95d114</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>JNJ</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" s="2" t="n">
+        <v>46325</v>
+      </c>
+      <c r="F35" t="n">
+        <v>273.2</v>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="H35" t="n">
+        <v>755.72</v>
+      </c>
+      <c r="I35" t="n">
+        <v>48.7</v>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L35" t="n">
+        <v>33.9</v>
+      </c>
+      <c r="M35" t="n">
+        <v>63.5</v>
+      </c>
+      <c r="N35" t="n">
+        <v>273.2</v>
+      </c>
+      <c r="O35" t="n">
+        <v>0.206</v>
+      </c>
+      <c r="P35" t="n">
+        <v>41.456753</v>
+      </c>
+      <c r="Q35" t="n">
+        <v>23.51552</v>
+      </c>
+      <c r="R35" t="n">
+        <v>5.36</v>
+      </c>
+      <c r="S35" t="n">
+        <v>0.019619</v>
+      </c>
+      <c r="T35" t="n">
+        <v>-0.959</v>
+      </c>
+      <c r="U35" t="inlineStr">
+        <is>
+          <t>Healthcare</t>
+        </is>
+      </c>
+      <c r="V35" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="W35" t="n">
+        <v>0.0498</v>
+      </c>
+      <c r="X35" t="inlineStr">
+        <is>
+          <t>fred</t>
+        </is>
+      </c>
+      <c r="Y35" t="inlineStr">
+        <is>
+          <t>e95d114</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" s="2" t="n">
+        <v>46325</v>
+      </c>
+      <c r="F36" t="n">
+        <v>161.57</v>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="H36" t="n">
+        <v>755.72</v>
+      </c>
+      <c r="I36" t="n">
+        <v>61.5</v>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L36" t="n">
+        <v>53.4</v>
+      </c>
+      <c r="M36" t="n">
+        <v>69.5</v>
+      </c>
+      <c r="N36" t="n">
+        <v>161.57</v>
+      </c>
+      <c r="O36" t="n">
+        <v>0.377</v>
+      </c>
+      <c r="P36" t="n">
+        <v>24.332832</v>
+      </c>
+      <c r="Q36" t="n">
+        <v>21.84701</v>
+      </c>
+      <c r="R36" t="n">
+        <v>4.35</v>
+      </c>
+      <c r="S36" t="n">
+        <v>0.026923</v>
+      </c>
+      <c r="T36" t="n">
+        <v>0.008</v>
+      </c>
+      <c r="U36" t="inlineStr">
+        <is>
+          <t>Consumer Defensive</t>
+        </is>
+      </c>
+      <c r="V36" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="W36" t="n">
+        <v>0.0498</v>
+      </c>
+      <c r="X36" t="inlineStr">
+        <is>
+          <t>fred</t>
+        </is>
+      </c>
+      <c r="Y36" t="inlineStr">
+        <is>
+          <t>e95d114</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>KO</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr"/>
+      <c r="E37" s="2" t="n">
+        <v>46325</v>
+      </c>
+      <c r="F37" t="n">
+        <v>94.08</v>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="H37" t="n">
+        <v>755.72</v>
+      </c>
+      <c r="I37" t="n">
+        <v>69.5</v>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="L37" t="n">
+        <v>69.5</v>
+      </c>
+      <c r="M37" t="n">
+        <v>69.5</v>
+      </c>
+      <c r="N37" t="n">
+        <v>94.08</v>
+      </c>
+      <c r="O37" t="n">
+        <v>0.318</v>
+      </c>
+      <c r="P37" t="n">
+        <v>28.252253</v>
+      </c>
+      <c r="Q37" t="n">
+        <v>26.703074</v>
+      </c>
+      <c r="R37" t="n">
+        <v>2.12</v>
+      </c>
+      <c r="S37" t="n">
+        <v>0.022534</v>
+      </c>
+      <c r="T37" t="n">
+        <v>0.083</v>
+      </c>
+      <c r="U37" t="inlineStr">
+        <is>
+          <t>Consumer Defensive</t>
+        </is>
+      </c>
+      <c r="V37" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="W37" t="n">
+        <v>0.0498</v>
+      </c>
+      <c r="X37" t="inlineStr">
+        <is>
+          <t>fred</t>
+        </is>
+      </c>
+      <c r="Y37" t="inlineStr">
+        <is>
+          <t>e95d114</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>XOM</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr"/>
+      <c r="E38" s="2" t="n">
+        <v>46325</v>
+      </c>
+      <c r="F38" t="n">
+        <v>187.25</v>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="H38" t="n">
+        <v>755.72</v>
+      </c>
+      <c r="I38" t="n">
+        <v>69.90000000000001</v>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L38" t="n">
+        <v>80.8</v>
+      </c>
+      <c r="M38" t="n">
+        <v>59</v>
+      </c>
+      <c r="N38" t="n">
+        <v>187.25</v>
+      </c>
+      <c r="O38" t="inlineStr"/>
+      <c r="P38" t="n">
+        <v>19.264402</v>
+      </c>
+      <c r="Q38" t="n">
+        <v>15.586917</v>
+      </c>
+      <c r="R38" t="n">
+        <v>4.12</v>
+      </c>
+      <c r="S38" t="n">
+        <v>0.022003</v>
+      </c>
+      <c r="T38" t="n">
+        <v>1.114</v>
+      </c>
+      <c r="U38" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="V38" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="W38" t="n">
+        <v>0.0498</v>
+      </c>
+      <c r="X38" t="inlineStr">
+        <is>
+          <t>fred</t>
+        </is>
+      </c>
+      <c r="Y38" t="inlineStr">
+        <is>
+          <t>e95d114</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>NKE</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr"/>
+      <c r="E39" s="2" t="n">
+        <v>46325</v>
+      </c>
+      <c r="F39" t="n">
+        <v>38.67</v>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="H39" t="n">
+        <v>755.72</v>
+      </c>
+      <c r="I39" t="n">
+        <v>47.6</v>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L39" t="n">
+        <v>45.2</v>
+      </c>
+      <c r="M39" t="n">
+        <v>50</v>
+      </c>
+      <c r="N39" t="n">
+        <v>38.67</v>
+      </c>
+      <c r="O39" t="n">
+        <v>1.099</v>
+      </c>
+      <c r="P39" t="n">
+        <v>18.591347</v>
+      </c>
+      <c r="Q39" t="n">
+        <v>24.835106</v>
+      </c>
+      <c r="R39" t="n">
+        <v>1.64</v>
+      </c>
+      <c r="S39" t="n">
+        <v>0.04241</v>
+      </c>
+      <c r="T39" t="n">
+        <v>-0.021</v>
+      </c>
+      <c r="U39" t="inlineStr">
+        <is>
+          <t>Consumer Cyclical</t>
+        </is>
+      </c>
+      <c r="V39" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="W39" t="n">
+        <v>0.0498</v>
+      </c>
+      <c r="X39" t="inlineStr">
+        <is>
+          <t>fred</t>
+        </is>
+      </c>
+      <c r="Y39" t="inlineStr">
+        <is>
+          <t>e95d114</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr"/>
+      <c r="E40" s="2" t="n">
+        <v>46325</v>
+      </c>
+      <c r="F40" t="n">
+        <v>399.81</v>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="H40" t="n">
+        <v>755.72</v>
+      </c>
+      <c r="I40" t="n">
+        <v>31.1</v>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="L40" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="M40" t="n">
+        <v>60.5</v>
+      </c>
+      <c r="N40" t="n">
+        <v>399.81</v>
+      </c>
+      <c r="O40" t="n">
+        <v>1.916</v>
+      </c>
+      <c r="P40" t="n">
+        <v>439.35162</v>
+      </c>
+      <c r="Q40" t="n">
+        <v>185.5</v>
+      </c>
+      <c r="R40" t="inlineStr"/>
+      <c r="S40" t="n">
+        <v>0</v>
+      </c>
+      <c r="T40" t="n">
+        <v>-0.436</v>
+      </c>
+      <c r="U40" t="inlineStr">
+        <is>
+          <t>Consumer Cyclical</t>
+        </is>
+      </c>
+      <c r="V40" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="W40" t="n">
+        <v>0.0498</v>
+      </c>
+      <c r="X40" t="inlineStr">
+        <is>
+          <t>fred</t>
+        </is>
+      </c>
+      <c r="Y40" t="inlineStr">
+        <is>
+          <t>e95d114</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>ASML.AS</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr"/>
+      <c r="E41" s="2" t="n">
+        <v>46325</v>
+      </c>
+      <c r="F41" t="n">
+        <v>1412.8</v>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="H41" t="n">
+        <v>755.72</v>
+      </c>
+      <c r="I41" t="n">
+        <v>42.8</v>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L41" t="n">
+        <v>31</v>
+      </c>
+      <c r="M41" t="n">
+        <v>54.5</v>
+      </c>
+      <c r="N41" t="n">
+        <v>1412.8</v>
+      </c>
+      <c r="O41" t="n">
+        <v>1.302</v>
+      </c>
+      <c r="P41" t="n">
+        <v>40.388794</v>
+      </c>
+      <c r="Q41" t="n">
+        <v>25.2606</v>
+      </c>
+      <c r="R41" t="n">
+        <v>7.52</v>
+      </c>
+      <c r="S41" t="n">
+        <v>0.005323</v>
+      </c>
+      <c r="T41" t="n">
+        <v>1.359</v>
+      </c>
+      <c r="U41" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="V41" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="W41" t="n">
+        <v>0.0498</v>
+      </c>
+      <c r="X41" t="inlineStr">
+        <is>
+          <t>fred</t>
+        </is>
+      </c>
+      <c r="Y41" t="inlineStr">
+        <is>
+          <t>e95d114</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>SAP.DE</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr"/>
+      <c r="E42" s="2" t="n">
+        <v>46325</v>
+      </c>
+      <c r="F42" t="n">
+        <v>211.25</v>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="H42" t="n">
+        <v>755.72</v>
+      </c>
+      <c r="I42" t="n">
+        <v>63.8</v>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="L42" t="n">
+        <v>64</v>
+      </c>
+      <c r="M42" t="n">
+        <v>63.5</v>
+      </c>
+      <c r="N42" t="n">
+        <v>211.25</v>
+      </c>
+      <c r="O42" t="n">
+        <v>0.758</v>
+      </c>
+      <c r="P42" t="n">
+        <v>30.571636</v>
+      </c>
+      <c r="Q42" t="n">
+        <v>24.925726</v>
+      </c>
+      <c r="R42" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="S42" t="n">
+        <v>0.011834</v>
+      </c>
+      <c r="T42" t="n">
+        <v>0.134</v>
+      </c>
+      <c r="U42" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="V42" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="W42" t="n">
+        <v>0.0498</v>
+      </c>
+      <c r="X42" t="inlineStr">
+        <is>
+          <t>fred</t>
+        </is>
+      </c>
+      <c r="Y42" t="inlineStr">
+        <is>
+          <t>e95d114</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>MC.PA</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr"/>
+      <c r="E43" s="2" t="n">
+        <v>46325</v>
+      </c>
+      <c r="F43" t="n">
+        <v>387</v>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="H43" t="n">
+        <v>755.72</v>
+      </c>
+      <c r="I43" t="n">
+        <v>46.4</v>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L43" t="n">
+        <v>48.7</v>
+      </c>
+      <c r="M43" t="n">
+        <v>44</v>
+      </c>
+      <c r="N43" t="n">
+        <v>387</v>
+      </c>
+      <c r="O43" t="n">
+        <v>0.879</v>
+      </c>
+      <c r="P43" t="n">
+        <v>17.784925</v>
+      </c>
+      <c r="Q43" t="n">
+        <v>16.031609</v>
+      </c>
+      <c r="R43" t="n">
+        <v>13</v>
+      </c>
+      <c r="S43" t="n">
+        <v>0.033592</v>
+      </c>
+      <c r="T43" t="n">
+        <v>0.008</v>
+      </c>
+      <c r="U43" t="inlineStr">
+        <is>
+          <t>Consumer Cyclical</t>
+        </is>
+      </c>
+      <c r="V43" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="W43" t="n">
+        <v>0.0498</v>
+      </c>
+      <c r="X43" t="inlineStr">
+        <is>
+          <t>fred</t>
+        </is>
+      </c>
+      <c r="Y43" t="inlineStr">
+        <is>
+          <t>e95d114</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>SAN.MC</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr"/>
+      <c r="E44" s="2" t="n">
+        <v>46325</v>
+      </c>
+      <c r="F44" t="n">
+        <v>10.118</v>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="H44" t="n">
+        <v>755.72</v>
+      </c>
+      <c r="I44" t="n">
+        <v>47</v>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L44" t="n">
+        <v>53.1</v>
+      </c>
+      <c r="M44" t="n">
+        <v>41</v>
+      </c>
+      <c r="N44" t="n">
+        <v>10.118</v>
+      </c>
+      <c r="O44" t="n">
+        <v>0.9419999999999999</v>
+      </c>
+      <c r="P44" t="n">
+        <v>11.118681</v>
+      </c>
+      <c r="Q44" t="n">
+        <v>8.084117000000001</v>
+      </c>
+      <c r="R44" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="S44" t="n">
+        <v>0.024708</v>
+      </c>
+      <c r="T44" t="n">
+        <v>0.052</v>
+      </c>
+      <c r="U44" t="inlineStr">
+        <is>
+          <t>Financial Services</t>
+        </is>
+      </c>
+      <c r="V44" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="W44" t="n">
+        <v>0.0498</v>
+      </c>
+      <c r="X44" t="inlineStr">
+        <is>
+          <t>fred</t>
+        </is>
+      </c>
+      <c r="Y44" t="inlineStr">
+        <is>
+          <t>e95d114</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>ITX.MC</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr"/>
+      <c r="E45" s="2" t="n">
+        <v>46325</v>
+      </c>
+      <c r="F45" t="n">
+        <v>56.14</v>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="H45" t="n">
+        <v>755.72</v>
+      </c>
+      <c r="I45" t="n">
+        <v>56</v>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L45" t="n">
+        <v>50.1</v>
+      </c>
+      <c r="M45" t="n">
+        <v>62</v>
+      </c>
+      <c r="N45" t="n">
+        <v>56.14</v>
+      </c>
+      <c r="O45" t="n">
+        <v>0.959</v>
+      </c>
+      <c r="P45" t="n">
+        <v>27.252428</v>
+      </c>
+      <c r="Q45" t="n">
+        <v>23.749693</v>
+      </c>
+      <c r="R45" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S45" t="n">
+        <v>0.011578</v>
+      </c>
+      <c r="T45" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="U45" t="inlineStr">
+        <is>
+          <t>Consumer Cyclical</t>
+        </is>
+      </c>
+      <c r="V45" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="W45" t="n">
+        <v>0.0498</v>
+      </c>
+      <c r="X45" t="inlineStr">
+        <is>
+          <t>fred</t>
+        </is>
+      </c>
+      <c r="Y45" t="inlineStr">
+        <is>
+          <t>e95d114</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>IBE.MC</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr"/>
+      <c r="E46" s="2" t="n">
+        <v>46325</v>
+      </c>
+      <c r="F46" t="n">
+        <v>22.18</v>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="H46" t="n">
+        <v>755.72</v>
+      </c>
+      <c r="I46" t="n">
+        <v>49.8</v>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L46" t="n">
+        <v>40.5</v>
+      </c>
+      <c r="M46" t="n">
+        <v>59</v>
+      </c>
+      <c r="N46" t="n">
+        <v>22.18</v>
+      </c>
+      <c r="O46" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="P46" t="n">
+        <v>29.972973</v>
+      </c>
+      <c r="Q46" t="n">
+        <v>19.912199</v>
+      </c>
+      <c r="R46" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="S46" t="n">
+        <v>0.030658</v>
+      </c>
+      <c r="T46" t="n">
+        <v>-0.134</v>
+      </c>
+      <c r="U46" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="V46" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="W46" t="n">
+        <v>0.0498</v>
+      </c>
+      <c r="X46" t="inlineStr">
+        <is>
+          <t>fred</t>
+        </is>
+      </c>
+      <c r="Y46" t="inlineStr">
+        <is>
+          <t>e95d114</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>BBVA.MC</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr"/>
+      <c r="E47" s="2" t="n">
+        <v>46325</v>
+      </c>
+      <c r="F47" t="n">
+        <v>21.06</v>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="H47" t="n">
+        <v>755.72</v>
+      </c>
+      <c r="I47" t="n">
+        <v>71.90000000000001</v>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L47" t="n">
+        <v>87.8</v>
+      </c>
+      <c r="M47" t="n">
+        <v>56</v>
+      </c>
+      <c r="N47" t="n">
+        <v>21.06</v>
+      </c>
+      <c r="O47" t="n">
+        <v>0.902</v>
+      </c>
+      <c r="P47" t="n">
+        <v>10.744898</v>
+      </c>
+      <c r="Q47" t="n">
+        <v>8.962846000000001</v>
+      </c>
+      <c r="R47" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="S47" t="n">
+        <v>0.046059</v>
+      </c>
+      <c r="T47" t="n">
+        <v>0.238</v>
+      </c>
+      <c r="U47" t="inlineStr">
+        <is>
+          <t>Financial Services</t>
+        </is>
+      </c>
+      <c r="V47" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="W47" t="n">
+        <v>0.0498</v>
+      </c>
+      <c r="X47" t="inlineStr">
+        <is>
+          <t>fred</t>
+        </is>
+      </c>
+      <c r="Y47" t="inlineStr">
+        <is>
+          <t>e95d114</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>TEF.MC</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr"/>
+      <c r="E48" s="2" t="n">
+        <v>46325</v>
+      </c>
+      <c r="F48" t="n">
+        <v>3.374</v>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="H48" t="n">
+        <v>755.72</v>
+      </c>
+      <c r="I48" t="n">
+        <v>69.7</v>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="L48" t="n">
+        <v>93.90000000000001</v>
+      </c>
+      <c r="M48" t="n">
+        <v>45.5</v>
+      </c>
+      <c r="N48" t="n">
+        <v>3.374</v>
+      </c>
+      <c r="O48" t="n">
+        <v>0.306</v>
+      </c>
+      <c r="P48" t="inlineStr"/>
+      <c r="Q48" t="n">
+        <v>8.577166999999999</v>
+      </c>
+      <c r="R48" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="S48" t="n">
+        <v>0.044458</v>
+      </c>
+      <c r="T48" t="inlineStr"/>
+      <c r="U48" t="inlineStr">
+        <is>
+          <t>Communication Services</t>
+        </is>
+      </c>
+      <c r="V48" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="W48" t="n">
+        <v>0.0498</v>
+      </c>
+      <c r="X48" t="inlineStr">
+        <is>
+          <t>fred</t>
+        </is>
+      </c>
+      <c r="Y48" t="inlineStr">
+        <is>
+          <t>e95d114</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>REP.MC</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr"/>
+      <c r="E49" s="2" t="n">
+        <v>46325</v>
+      </c>
+      <c r="F49" t="n">
+        <v>30.73</v>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="H49" t="n">
+        <v>755.72</v>
+      </c>
+      <c r="I49" t="n">
+        <v>67.7</v>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="L49" t="n">
+        <v>71.8</v>
+      </c>
+      <c r="M49" t="n">
+        <v>63.5</v>
+      </c>
+      <c r="N49" t="n">
+        <v>30.73</v>
+      </c>
+      <c r="O49" t="n">
+        <v>-0.12</v>
+      </c>
+      <c r="P49" t="n">
+        <v>5.458259</v>
+      </c>
+      <c r="Q49" t="n">
+        <v>6.836926</v>
+      </c>
+      <c r="R49" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="S49" t="n">
+        <v>0.034169</v>
+      </c>
+      <c r="T49" t="n">
+        <v>4.224</v>
+      </c>
+      <c r="U49" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="V49" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="W49" t="n">
+        <v>0.0498</v>
+      </c>
+      <c r="X49" t="inlineStr">
+        <is>
+          <t>fred</t>
+        </is>
+      </c>
+      <c r="Y49" t="inlineStr">
+        <is>
+          <t>e95d114</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>AIR.PA</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr"/>
+      <c r="E50" s="2" t="n">
+        <v>46325</v>
+      </c>
+      <c r="F50" t="n">
+        <v>192.4</v>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="H50" t="n">
+        <v>755.72</v>
+      </c>
+      <c r="I50" t="n">
+        <v>72.09999999999999</v>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L50" t="n">
+        <v>82.2</v>
+      </c>
+      <c r="M50" t="n">
+        <v>62</v>
+      </c>
+      <c r="N50" t="n">
+        <v>192.4</v>
+      </c>
+      <c r="O50" t="n">
+        <v>0.887</v>
+      </c>
+      <c r="P50" t="n">
+        <v>25.619173</v>
+      </c>
+      <c r="Q50" t="n">
+        <v>22.183125</v>
+      </c>
+      <c r="R50" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="S50" t="n">
+        <v>0.016632</v>
+      </c>
+      <c r="T50" t="n">
+        <v>0.206</v>
+      </c>
+      <c r="U50" t="inlineStr">
+        <is>
+          <t>Industrials</t>
+        </is>
+      </c>
+      <c r="V50" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="W50" t="n">
+        <v>0.0498</v>
+      </c>
+      <c r="X50" t="inlineStr">
+        <is>
+          <t>fred</t>
+        </is>
+      </c>
+      <c r="Y50" t="inlineStr">
+        <is>
+          <t>e95d114</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>SIE.DE</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr"/>
+      <c r="E51" s="2" t="n">
+        <v>46325</v>
+      </c>
+      <c r="F51" t="n">
+        <v>265.65</v>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="H51" t="n">
+        <v>755.72</v>
+      </c>
+      <c r="I51" t="n">
+        <v>47.9</v>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L51" t="n">
+        <v>35.3</v>
+      </c>
+      <c r="M51" t="n">
+        <v>60.5</v>
+      </c>
+      <c r="N51" t="n">
+        <v>265.65</v>
+      </c>
+      <c r="O51" t="n">
+        <v>1.295</v>
+      </c>
+      <c r="P51" t="n">
+        <v>26.564999</v>
+      </c>
+      <c r="Q51" t="n">
+        <v>20.424671</v>
+      </c>
+      <c r="R51" t="n">
+        <v>5.35</v>
+      </c>
+      <c r="S51" t="n">
+        <v>0.020139</v>
+      </c>
+      <c r="T51" t="n">
+        <v>0.128</v>
+      </c>
+      <c r="U51" t="inlineStr">
+        <is>
+          <t>Industrials</t>
+        </is>
+      </c>
+      <c r="V51" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="W51" t="n">
+        <v>0.0498</v>
+      </c>
+      <c r="X51" t="inlineStr">
+        <is>
+          <t>fred</t>
+        </is>
+      </c>
+      <c r="Y51" t="inlineStr">
+        <is>
+          <t>e95d114</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Y26"/>
+  <autoFilter ref="A1:Y51"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>